<commit_message>
AI steps: figures as requests of their own, collected as figure designs, drawn by tfl_ai_run()
figure-1 ... with the figure's shell; the answer (a figure design) checked and
written as the report file in the design's form (round-trips to the same
design); tfl_ai_run() draws it with tfl_fig_design_code() (PNG, RTF). A type
column (table/figure) in the requests and reports, png in the run's reports.
The example workbook has a KM figure, with a stored answer.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/ai/example/onco_toc_shell.xlsx
+++ b/inst/ai/example/onco_toc_shell.xlsx
@@ -9,13 +9,14 @@
     <sheet name="TOC" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="T14.1.1" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="T14.2.1" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Safety" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="F14.2.2" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Safety" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="97">
   <si>
     <t xml:space="preserve">XYZ-ONC-01 Table of Contents (draft 0.2)</t>
   </si>
@@ -71,6 +72,18 @@
     <t xml:space="preserve">t_orr.sas</t>
   </si>
   <si>
+    <t xml:space="preserve">F-14-2-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaplan-Meier Plot of Overall Survival</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_km_os.sas</t>
+  </si>
+  <si>
     <t xml:space="preserve">14.3 Safety Data</t>
   </si>
   <si>
@@ -222,6 +235,27 @@
   </si>
   <si>
     <t xml:space="preserve">95% CI: Clopper-Pearson exact confidence interval.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure 14.2.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Kaplan-Meier curves, one per arm: Drug X, Control]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X axis: Time (Months), from 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y axis: Survival Probability, 0 to 1 by 0.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Censored subjects marked on the curves (+)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legend inside the plot, top right</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overall survival: ADTTE, PARAMCD = OS; censored when CNSR = 1.</t>
   </si>
   <si>
     <t xml:space="preserve">Table 14.3.1</t>
@@ -721,53 +755,70 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="E8" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E9" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
       </c>
       <c r="E10" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -792,7 +843,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2">
@@ -802,7 +853,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">
@@ -810,202 +861,202 @@
         <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D11" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B13" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D13" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B16" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D17" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B19" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C19" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D19" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B20" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C20" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D20" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1030,7 +1081,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2">
@@ -1040,7 +1091,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5">
@@ -1048,118 +1099,118 @@
         <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C10" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C15" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1177,6 +1228,79 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
+    <col min="1" max="1" width="70.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:D3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
     <col min="1" max="1" width="44.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="14.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="14.71" hidden="0" customWidth="1"/>
@@ -1186,130 +1310,130 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C10" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22">
@@ -1317,13 +1441,13 @@
         <v>6</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D22" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E22" t="s">
         <v>6</v>
@@ -1331,102 +1455,102 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="D23" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="E23" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="B25" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C25" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D25" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E25" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="B26" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C26" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D26" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E26" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="B28" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C28" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D28" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E28" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="B29" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C29" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D29" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E29" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>